<commit_message>
Orden de data cleaning y  actualización de archivos
</commit_message>
<xml_diff>
--- a/df_finall.xlsx
+++ b/df_finall.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://molt246-my.sharepoint.com/personal/lauras_molt_com_co/Documents/Documentos/GitHub/Costo mano de obra/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="38" documentId="11_4331D2B1D3F0D76CDB382F11595ED87656CAB93A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{6CB6203E-60B3-4B39-9DA2-77926555193A}"/>
+  <xr:revisionPtr revIDLastSave="41" documentId="11_4331D2B1D3F0D76CDB382F11595ED87656CAB93A" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2709A667-C638-467C-AF6B-0C0CAD0A37CD}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -5032,10 +5032,6 @@
 </styleSheet>
 </file>
 
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
-</file>
-
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{6B3035B8-B8CB-4713-A65B-B87037BD2A17}" name="Tabla1" displayName="Tabla1" ref="A1:W471" totalsRowCount="1" headerRowDxfId="16" headerRowBorderDxfId="15" tableBorderDxfId="14">
   <autoFilter ref="A1:W470" xr:uid="{6B3035B8-B8CB-4713-A65B-B87037BD2A17}"/>
@@ -5059,19 +5055,19 @@
     <tableColumn id="14" xr3:uid="{284E1164-5CA7-4C95-BD15-DB5A407B9A06}" name="Num OS"/>
     <tableColumn id="15" xr3:uid="{68F59A93-1878-4086-B3DF-5DA83BBD5780}" name="Nombre del Comercial"/>
     <tableColumn id="16" xr3:uid="{36272DC0-582E-44BA-A350-C5B36EAD2D62}" name="Categoría"/>
-    <tableColumn id="17" xr3:uid="{8F40440C-0351-4230-B60A-699199CC9FEC}" name="Total Precio Sin IVA" dataDxfId="13" totalsRowDxfId="6"/>
-    <tableColumn id="18" xr3:uid="{F235B113-E95E-42BB-A570-03C646EBE0EA}" name="costo_antes_iva" dataDxfId="12" totalsRowDxfId="5"/>
-    <tableColumn id="19" xr3:uid="{4CCCE524-F3D6-447E-9614-684F287EC8ED}" name="OS-Valor Unitario" dataDxfId="11" totalsRowDxfId="4"/>
-    <tableColumn id="20" xr3:uid="{92D6C706-19B2-41C1-960F-0F19A34EFF7A}" name="Diferencia valor unitario" dataDxfId="10" totalsRowDxfId="3">
+    <tableColumn id="17" xr3:uid="{8F40440C-0351-4230-B60A-699199CC9FEC}" name="Total Precio Sin IVA" dataDxfId="13" totalsRowDxfId="12"/>
+    <tableColumn id="18" xr3:uid="{F235B113-E95E-42BB-A570-03C646EBE0EA}" name="costo_antes_iva" dataDxfId="11" totalsRowDxfId="10"/>
+    <tableColumn id="19" xr3:uid="{4CCCE524-F3D6-447E-9614-684F287EC8ED}" name="OS-Valor Unitario" dataDxfId="9" totalsRowDxfId="8"/>
+    <tableColumn id="20" xr3:uid="{92D6C706-19B2-41C1-960F-0F19A34EFF7A}" name="Diferencia valor unitario" dataDxfId="7" totalsRowDxfId="6">
       <calculatedColumnFormula>Tabla1[[#This Row],[OS-Valor Unitario]]-Tabla1[[#This Row],[costo_antes_iva]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="21" xr3:uid="{1AF8AD52-D22C-417F-A041-6FB246F72068}" name="Valor total OS" dataDxfId="9" totalsRowDxfId="2">
+    <tableColumn id="21" xr3:uid="{1AF8AD52-D22C-417F-A041-6FB246F72068}" name="Valor total OS" dataDxfId="5" totalsRowDxfId="4">
       <calculatedColumnFormula>Tabla1[[#This Row],[OS-Valor Unitario]]*Tabla1[[#This Row],[OS-Cantidad]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="22" xr3:uid="{DF14BE5A-2081-4559-848E-5D50DB13DCCD}" name="valor total op" dataDxfId="8" totalsRowDxfId="1">
+    <tableColumn id="22" xr3:uid="{DF14BE5A-2081-4559-848E-5D50DB13DCCD}" name="valor total op" dataDxfId="3" totalsRowDxfId="2">
       <calculatedColumnFormula>Tabla1[[#This Row],[costo_antes_iva]]*Tabla1[[#This Row],[OS-Cantidad]]</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="23" xr3:uid="{9F2434E0-B8A1-476A-BDBE-31342159F154}" name="Diferencia" totalsRowFunction="sum" dataDxfId="7" totalsRowDxfId="0">
+    <tableColumn id="23" xr3:uid="{9F2434E0-B8A1-476A-BDBE-31342159F154}" name="Diferencia" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0">
       <calculatedColumnFormula>Tabla1[[#This Row],[Valor total OS]]-Tabla1[[#This Row],[valor total op]]</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -5375,7 +5371,7 @@
     <col min="11" max="11" width="19.5546875" customWidth="1"/>
     <col min="12" max="12" width="10" customWidth="1"/>
     <col min="13" max="13" width="13.44140625" customWidth="1"/>
-    <col min="14" max="14" width="40.6640625" customWidth="1"/>
+    <col min="14" max="14" width="41.33203125" customWidth="1"/>
     <col min="15" max="15" width="21.5546875" customWidth="1"/>
     <col min="16" max="16" width="10.88671875" customWidth="1"/>
     <col min="17" max="17" width="19.21875" style="4" customWidth="1"/>

</xml_diff>